<commit_message>
refactor(blog): change all article title prefixes from 【飛田新地 求人】 to 【飛田新地】
</commit_message>
<xml_diff>
--- a/public/tobitashinchi_articles.xlsx
+++ b/public/tobitashinchi_articles.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】仕事内容を徹底解説！特別な技術は一切不要！完全受け身で未経験者が即日デビューできる理由</t>
+          <t>【飛田新地】仕事内容を徹底解説！特別な技術は一切不要！完全受け身で未経験者が即日デビューできる理由</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】給料システム徹底解説！15分5,000円の仕組みと計算式・全額日払いで高収入が残る理由</t>
+          <t>【飛田新地】給料システム徹底解説！15分5,000円の仕組みと計算式・全額日払いで高収入が残る理由</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】身バレ・顔バレ防止の極意！会社や家族に100%知られない！現役キャストが実践する8大対策</t>
+          <t>【飛田新地】身バレ・顔バレ防止の極意！会社や家族に100%知られない！現役キャストが実践する8大対策</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】駅近マンション寮完備！家具家電付き・即日入居OK！出稼ぎ＆一人暮らしに嬉しい快適個室寮</t>
+          <t>【飛田新地】駅近マンション寮完備！家具家電付き・即日入居OK！出稼ぎ＆一人暮らしに嬉しい快適個室寮</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】応募資格・面接の必要書類！本籍地記載の住民票が必須な理由と採用ポイント</t>
+          <t>【飛田新地】応募資格・面接の必要書類！本籍地記載の住民票が必須な理由と採用ポイント</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】体験入店と面接の流れ！喫茶店面接から即日退店ルール・全額日払いまでの完全手順</t>
+          <t>【飛田新地】体験入店と面接の流れ！喫茶店面接から即日退店ルール・全額日払いまでの完全手順</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】本音で暴露！飛田新地で働くメリットとデメリット！風俗未経験者が知るべき真実</t>
+          <t>【飛田新地】本音で暴露！飛田新地で働くメリットとデメリット！風俗未経験者が知るべき真実</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】メイン通りと青春通りの違い！採用基準・ルックス・平均日給と働きやすさを徹底比較</t>
+          <t>【飛田新地】メイン通りと青春通りの違い！採用基準・ルックス・平均日給と働きやすさを徹底比較</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】衛生管理・性病予防の徹底！キスNG・完全ゴム着用！女の子の体を守る飛田新地の安心衛生ルール</t>
+          <t>【飛田新地】衛生管理・性病予防の徹底！キスNG・完全ゴム着用！女の子の体を守る飛田新地の安心衛生ルール</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】シフト・短時間勤務の働き方！昼番・夜番の2交代制と固定シフトで賢く稼ぐコツ</t>
+          <t>【飛田新地】シフト・短時間勤務の働き方！昼番・夜番の2交代制と固定シフトで賢く稼ぐコツ</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】最短1ヶ月から！短期集中でがっつり貯金！「今すぐお金が必要」を叶える短期稼働のススメ</t>
+          <t>【飛田新地】最短1ヶ月から！短期集中でがっつり貯金！「今すぐお金が必要」を叶える短期稼働のススメ</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】料亭の安全管理！飛田新地の客層が良い理由！お店のスタッフが徹底する「女の子最優先」の警備体制</t>
+          <t>【飛田新地】料亭の安全管理！飛田新地の客層が良い理由！お店のスタッフが徹底する「女の子最優先」の警備体制</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】和装・メイク術！自分に一番似合うスタイルは？無料レンタル浴衣・着物とお仕事メイクのコツ</t>
+          <t>【飛田新地】和装・メイク術！自分に一番似合うスタイルは？無料レンタル浴衣・着物とお仕事メイクのコツ</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】週1日・週末だけOK！OL・会社員や学生さん必見！お昼だけ・週末だけの掛け持ちシフト例</t>
+          <t>【飛田新地】週1日・週末だけOK！OL・会社員や学生さん必見！お昼だけ・週末だけの掛け持ちシフト例</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】心に寄り添うサポート！悩みは一人で抱え込まないで！現役キャストが教える女性スタッフの頼り方</t>
+          <t>【飛田新地】心に寄り添うサポート！悩みは一人で抱え込まないで！現役キャストが教える女性スタッフの頼り方</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】徹底分析！飛田新地で働きたい女性が検索するワードとは？不安と疑問を先回り解決！</t>
+          <t>【飛田新地】徹底分析！飛田新地で働きたい女性が検索するワードとは？不安と疑問を先回り解決！</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】完全密着！飛田新地の1日！出勤からお仕事、退勤までのリアルな流れをレポート</t>
+          <t>【飛田新地】完全密着！飛田新地の1日！出勤からお仕事、退勤までのリアルな流れをレポート</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】おばちゃんは怖い？味方？飛田新地「売り子さん」の本当の役割と良好な関係作りのコツ</t>
+          <t>【飛田新地】おばちゃんは怖い？味方？飛田新地「売り子さん」の本当の役割と良好な関係作りのコツ</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】和装マジック！自分史上いちばん可愛くなれる！貸出衣装（着物・浴衣）とヘアメイクのこだわり</t>
+          <t>【飛田新地】和装マジック！自分史上いちばん可愛くなれる！貸出衣装（着物・浴衣）とヘアメイクのこだわり</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】身バレ対策の極意！家族・友達・会社に100%知られずに働き続けるための5つの鉄則</t>
+          <t>【飛田新地】身バレ対策の極意！家族・友達・会社に100%知られずに働き続けるための5つの鉄則</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】年齢・ルックスのリアル！18歳から40代まで！飛田新地で求められるキャストの条件とは？</t>
+          <t>【飛田新地】年齢・ルックスのリアル！18歳から40代まで！飛田新地で求められるキャストの条件とは？</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】防犯・安全マニュアル！お酒不要でトラブルなし！女の子を守り抜く飛田新地の鉄壁セキュリティ</t>
+          <t>【飛田新地】防犯・安全マニュアル！お酒不要でトラブルなし！女の子を守り抜く飛田新地の鉄壁セキュリティ</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】副業・OL・学生さんへ！週1日・短時間勤務でも効率的に高収入を稼ぐ賢いシフト設計テクニック</t>
+          <t>【飛田新地】副業・OL・学生さんへ！週1日・短時間勤務でも効率的に高収入を稼ぐ賢いシフト設計テクニック</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】体験入店の完全ガイド！面接の服装から必要な持ち物、当日の流れまでを徹底解説！</t>
+          <t>【飛田新地】体験入店の完全ガイド！面接の服装から必要な持ち物、当日の流れまでを徹底解説！</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】メンタルケア！ストレスを溜めない！飛田新地で心穏やかに＆笑顔で働き続けるためのマインドハック</t>
+          <t>【飛田新地】メンタルケア！ストレスを溜めない！飛田新地で心穏やかに＆笑顔で働き続けるためのマインドハック</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】未経験から人気キャストへ！指名・リピートが途切れない！誰でもすぐに実践できる3つの極秘接客術</t>
+          <t>【飛田新地】未経験から人気キャストへ！指名・リピートが途切れない！誰でもすぐに実践できる3つの極秘接客術</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】憧れの美容代に！飛田新地バイトで叶える「自分磨き」＆ハイブランド購入計画</t>
+          <t>【飛田新地】憧れの美容代に！飛田新地バイトで叶える「自分磨き」＆ハイブランド購入計画</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】女子大生・専門学生必見！親に内緒で卒業旅行＆奨学金返済！学業と両立するスマートな働き方</t>
+          <t>【飛田新地】女子大生・専門学生必見！親に内緒で卒業旅行＆奨学金返済！学業と両立するスマートな働き方</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】お給料の使い道！20代で1000万円貯めた女の子の貯金術とモチベーション維持の秘訣</t>
+          <t>【飛田新地】お給料の使い道！20代で1000万円貯めた女の子の貯金術とモチベーション維持の秘訣</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】友達同士の応募もOK！1人じゃ不安なあなたへ！友達と一緒に面接・体験入店するメリット</t>
+          <t>【飛田新地】友達同士の応募もOK！1人じゃ不安なあなたへ！友達と一緒に面接・体験入店するメリット</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】大阪・天王寺エリア魅力！お仕事前後に楽しめる！女子に大人気のおしゃれカフェ＆お買い物スポット</t>
+          <t>【飛田新地】大阪・天王寺エリア魅力！お仕事前後に楽しめる！女子に大人気のおしゃれカフェ＆お買い物スポット</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】入店祝い金・各種手当！求人サイトでよく見る「入店お祝い金」って本当にもらえる？お得な待遇の裏側</t>
+          <t>【飛田新地】入店祝い金・各種手当！求人サイトでよく見る「入店お祝い金」って本当にもらえる？お得な待遇の裏側</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】20代前半の強み！未経験から最速で稼ぎ頭になるための、愛され笑顔と愛嬌の磨き方</t>
+          <t>【飛田新地】20代前半の強み！未経験から最速で稼ぎ頭になるための、愛され笑顔と愛嬌の磨き方</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】20代後半からのリスタート！「今さら遅い？」なんてない！大人の色気と落ち着きで稼ぐノウハウ</t>
+          <t>【飛田新地】20代後半からのリスタート！「今さら遅い？」なんてない！大人の色気と落ち着きで稼ぐノウハウ</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】自立した女性へ！飛田新地のバイトをステップアップに！将来起業・独立したい夢を叶える資金作り</t>
+          <t>【飛田新地】自立した女性へ！飛田新地のバイトをステップアップに！将来起業・独立したい夢を叶える資金作り</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】面接の裏ワザ！不採用にならないために！面接官が思わず「明日から来てほしい！」と惹かれるアピール方法</t>
+          <t>【飛田新地】面接の裏ワザ！不採用にならないために！面接官が思わず「明日から来てほしい！」と惹かれるアピール方法</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】寮生活のリアル！飛田新地周辺の「マンション寮」はどんな感じ？家具・家電付きで即入居可能な秘密</t>
+          <t>【飛田新地】寮生活のリアル！飛田新地周辺の「マンション寮」はどんな感じ？家具・家電付きで即入居可能な秘密</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】お昼のシフトがアツい！12:00〜18:00の昼勤務で効率よく稼げる理由とメリット</t>
+          <t>【飛田新地】お昼のシフトがアツい！12:00〜18:00の昼勤務で効率よく稼げる理由とメリット</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】心と体のセルフケア！お仕事の疲れを翌日に残さない！現役キャスト愛用のデトックス＆リラックス法</t>
+          <t>【飛田新地】心と体のセルフケア！お仕事の疲れを翌日に残さない！現役キャスト愛用のデトックス＆リラックス法</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】和装が初めてでも安心！5分でパッと着こなせる！お店で用意している簡単で可愛い着物・浴衣の仕組み</t>
+          <t>【飛田新地】和装が初めてでも安心！5分でパッと着こなせる！お店で用意している簡単で可愛い着物・浴衣の仕組み</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】キャバクラ・風俗との違い！夜職未経験者が「飛田新地が一番働きやすい」と口を揃える納得の理由</t>
+          <t>【飛田新地】キャバクラ・風俗との違い！夜職未経験者が「飛田新地が一番働きやすい」と口を揃える納得の理由</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】20代のための税金対策！年間いくらから納税が必要？税務署からお尋ねが来ないための基礎知識</t>
+          <t>【飛田新地】20代のための税金対策！年間いくらから納税が必要？税務署からお尋ねが来ないための基礎知識</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】モチベーションを保つコツ！「なんとなく勤務」はもったいない！夢を最速で叶える目標金額のロードマップ</t>
+          <t>【飛田新地】モチベーションを保つコツ！「なんとなく勤務」はもったいない！夢を最速で叶える目標金額のロードマップ</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】履歴書不要・即日体験！持ち物はスマホと身分証だけ！今週末にでもスタートできる超スピード体験入店</t>
+          <t>【飛田新地】履歴書不要・即日体験！持ち物はスマホと身分証だけ！今週末にでもスタートできる超スピード体験入店</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】スタッフって怖いの？！「飛田新地求人」直営料亭グループのスタッフがとにかく優しくてアットホームな理由</t>
+          <t>【飛田新地】スタッフって怖いの？！「飛田新地求人」直営料亭グループのスタッフがとにかく優しくてアットホームな理由</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】短期でサクッと！リゾートバイト感覚で大阪・飛田新地へ！1ヶ月限定で賢く稼ぐ地方女子の選択肢</t>
+          <t>【飛田新地】短期でサクッと！リゾートバイト感覚で大阪・飛田新地へ！1ヶ月限定で賢く稼ぐ地方女子の選択肢</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】これで安心！飛田新地で身バレせずに働く！徹底したプライバシー保護の秘訣</t>
+          <t>【飛田新地】これで安心！飛田新地で身バレせずに働く！徹底したプライバシー保護の秘訣</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】安心！飛田新地で身バレが不安なあなたへ！プロが教える徹底対策4選</t>
+          <t>【飛田新地】安心！飛田新地で身バレが不安なあなたへ！プロが教える徹底対策4選</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】身バレ防止の秘訣！飛田新地で安心して働く！プライバシーを守る5つの方法</t>
+          <t>【飛田新地】身バレ防止の秘訣！飛田新地で安心して働く！プライバシーを守る5つの方法</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】日給10万円も夢じゃない！飛田新地の給料システムを徹底解説！稼ぎの秘密を大公開</t>
+          <t>【飛田新地】日給10万円も夢じゃない！飛田新地の給料システムを徹底解説！稼ぎの秘密を大公開</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】飛田新地のお仕事ってどんな感じ？未経験さんが知っておきたい「お仕事の一日の流れ」</t>
+          <t>【飛田新地】飛田新地のお仕事ってどんな感じ？未経験さんが知っておきたい「お仕事の一日の流れ」</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】身バレ徹底ガード！飛田新地で安心して働く！プライバシー保護の秘訣とお店のサポート</t>
+          <t>【飛田新地】身バレ徹底ガード！飛田新地で安心して働く！プライバシー保護の秘訣とお店のサポート</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】日払いOK？！飛田新地の給料システムを徹底解説！未経験でも高収入の秘密とは？</t>
+          <t>【飛田新地】日払いOK？！飛田新地の給料システムを徹底解説！未経験でも高収入の秘密とは？</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】初めてでも大丈夫！飛田新地のお仕事ってどんな感じ？未経験さん向け1日の流れと安心ポイント</t>
+          <t>【飛田新地】初めてでも大丈夫！飛田新地のお仕事ってどんな感じ？未経験さん向け1日の流れと安心ポイント</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】「もしかしてバレる？」飛田新地で安心して働く！身バレ防止の徹底ガイド</t>
+          <t>【飛田新地】「もしかしてバレる？」飛田新地で安心して働く！身バレ防止の徹底ガイド</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】飛田新地のお給料システム徹底解説！未経験でも安心の高収入を実現する秘訣</t>
+          <t>【飛田新地】飛田新地のお給料システム徹底解説！未経験でも安心の高収入を実現する秘訣</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】完全ガイド！飛田新地未経験者が安心する、お仕事の流れと「体入」のすべて</t>
+          <t>【飛田新地】完全ガイド！飛田新地未経験者が安心する、お仕事の流れと「体入」のすべて</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】カフェで気軽に相談！対面・LINEでOK！飛田新地の不安を全部解消する個別カウンセリング</t>
+          <t>【飛田新地】カフェで気軽に相談！対面・LINEでOK！飛田新地の不安を全部解消する個別カウンセリング</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】完全無料！手ぶらでOK！お店で借りられるメイク道具＆ドレス・和装の充実サポート</t>
+          <t>【飛田新地】完全無料！手ぶらでOK！お店で借りられるメイク道具＆ドレス・和装の充実サポート</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】通勤・アクセス快適！天王寺・難波からすぐ！飛田新地のお仕事への通いやすさをチェック</t>
+          <t>【飛田新地】通勤・アクセス快適！天王寺・難波からすぐ！飛田新地のお仕事への通いやすさをチェック</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】貯金スピード10倍？！短期間で目標額を達成するための目標設定と資金計画シート</t>
+          <t>【飛田新地】貯金スピード10倍？！短期間で目標額を達成するための目標設定と資金計画シート</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】自分磨き・美容代手当！働くだけで綺麗になれる！美容サロン提携＆自分投資の極意</t>
+          <t>【飛田新地】自分磨き・美容代手当！働くだけで綺麗になれる！美容サロン提携＆自分投資の極意</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr">
@@ -3878,7 +3878,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】心穏やかに働く！お仕事後のリフレッシュ法と無理なく長く続けるメンタルコンディショニング</t>
+          <t>【飛田新地】心穏やかに働く！お仕事後のリフレッシュ法と無理なく長く続けるメンタルコンディショニング</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】深夜タクシー代支給・送りあり！終電後も安全帰宅！夜シフトの女の子を守る送迎システム</t>
+          <t>【飛田新地】深夜タクシー代支給・送りあり！終電後も安全帰宅！夜シフトの女の子を守る送迎システム</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
@@ -3984,7 +3984,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】SNS・身バレ対策完璧！Instagram・TikTokの鍵アカウント運用とお顔非公開徹底ルール</t>
+          <t>【飛田新地】SNS・身バレ対策完璧！Instagram・TikTokの鍵アカウント運用とお顔非公開徹底ルール</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】地方出稼ぎ・短期集中！往復交通費全額支給＆快適ホテル・個室寮でサクッと稼ぐ出張スタイル</t>
+          <t>【飛田新地】地方出稼ぎ・短期集中！往復交通費全額支給＆快適ホテル・個室寮でサクッと稼ぐ出張スタイル</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】完全自由シフト制！週1日・3時間〜OK！自分のライフスタイルを崩さずに高収入を得るコツ</t>
+          <t>【飛田新地】完全自由シフト制！週1日・3時間〜OK！自分のライフスタイルを崩さずに高収入を得るコツ</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -4143,7 +4143,7 @@
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】大阪グルメ＆観光スポット！お仕事終わりに立ち寄りたい！天王寺・新世界・難波のおすすめスポット</t>
+          <t>【飛田新地】大阪グルメ＆観光スポット！お仕事終わりに立ち寄りたい！天王寺・新世界・難波のおすすめスポット</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】季節のおすすめ着物スタイル！春夏秋冬で楽しむ料亭のお着物・和装コーディネート術</t>
+          <t>【飛田新地】季節のおすすめ着物スタイル！春夏秋冬で楽しむ料亭のお着物・和装コーディネート術</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】シフト管理アプリ＆スケジュール管理！学業・本業と両立する賢いスケジュール帳の作り方</t>
+          <t>【飛田新地】シフト管理アプリ＆スケジュール管理！学業・本業と両立する賢いスケジュール帳の作り方</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】友達同士の応募大歓迎！一緒にお店を選べる「友達ペア紹介」と安心サポート</t>
+          <t>【飛田新地】友達同士の応募大歓迎！一緒にお店を選べる「友達ペア紹介」と安心サポート</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】自分へのご褒美＆モチベーション！目標達成ごとに自分を褒める「プチご褒美」習慣</t>
+          <t>【飛田新地】自分へのご褒美＆モチベーション！目標達成ごとに自分を褒める「プチご褒美」習慣</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
@@ -4408,7 +4408,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】夜の静かなプライベート時間！お仕事後の上質な睡眠＆おうち時間の過ごし方</t>
+          <t>【飛田新地】夜の静かなプライベート時間！お仕事後の上質な睡眠＆おうち時間の過ごし方</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】ノーファンデでも美肌見え！接客で映えるスキンケア＆ツヤ肌づくり徹底講座</t>
+          <t>【飛田新地】ノーファンデでも美肌見え！接客で映えるスキンケア＆ツヤ肌づくり徹底講座</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】自己肯定感がアップする！飛田新地のお仕事で変わった「私の自信と将来の夢」</t>
+          <t>【飛田新地】自己肯定感がアップする！飛田新地のお仕事で変わった「私の自信と将来の夢」</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -4567,7 +4567,7 @@
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】憧れの海外旅行・留学資金！短期間で目標額を貯めて海外へ羽ばたくキャストの資金活用術</t>
+          <t>【飛田新地】憧れの海外旅行・留学資金！短期間で目標額を貯めて海外へ羽ばたくキャストの資金活用術</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
@@ -4620,7 +4620,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】お休み日の至福ケア！バスタイムで疲れをリセット！バスソルト＆泡風呂の癒やし習慣</t>
+          <t>【飛田新地】お休み日の至福ケア！バスタイムで疲れをリセット！バスソルト＆泡風呂の癒やし習慣</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -4673,7 +4673,7 @@
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】カフェ巡り＆映えスイーツ！稼いだお金で休日を楽しむ！天王寺・心斎橋のおすすめカフェ5選</t>
+          <t>【飛田新地】カフェ巡り＆映えスイーツ！稼いだお金で休日を楽しむ！天王寺・心斎橋のおすすめカフェ5選</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】ほっと一息朝時間！出勤前や休日の朝を優雅に過ごすモーニングルーティン</t>
+          <t>【飛田新地】ほっと一息朝時間！出勤前や休日の朝を優雅に過ごすモーニングルーティン</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -4779,7 +4779,7 @@
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】季節のお花でお部屋を飾る！お部屋の雰囲気を明るくして運気を上げるプチインテリア術</t>
+          <t>【飛田新地】季節のお花でお部屋を飾る！お部屋の雰囲気を明るくして運気を上げるプチインテリア術</t>
         </is>
       </c>
       <c r="C81" s="9" t="inlineStr">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】銀行口座・手渡し徹底比較！日払い現金を安全に保管・口座管理するコツ</t>
+          <t>【飛田新地】銀行口座・手渡し徹底比較！日払い現金を安全に保管・口座管理するコツ</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】夜空を見上げてリセット！出勤後のナイトルーティンと心を落ち着かせる夜の過ごし方</t>
+          <t>【飛田新地】夜空を見上げてリセット！出勤後のナイトルーティンと心を落ち着かせる夜の過ごし方</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】料亭文化の奥深さ！伝統と品格を感じる「和の所作・マナー」が自然と身につく理由</t>
+          <t>【飛田新地】料亭文化の奥深さ！伝統と品格を感じる「和の所作・マナー」が自然と身につく理由</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -4991,7 +4991,7 @@
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】おうち時間を快適に！お仕事の疲れを癒やすルームウェア＆おうちリラクゼーション</t>
+          <t>【飛田新地】おうち時間を快適に！お仕事の疲れを癒やすルームウェア＆おうちリラクゼーション</t>
         </is>
       </c>
       <c r="C85" s="9" t="inlineStr">
@@ -5044,7 +5044,7 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】手鏡を見るたび笑顔に！お仕事を通して「自分の顔や雰囲気が好きになれた」秘密</t>
+          <t>【飛田新地】手鏡を見るたび笑顔に！お仕事を通して「自分の顔や雰囲気が好きになれた」秘密</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】思い出を形に残す写真旅！カメラや旅行趣味を楽しむ現役キャストのライフスタイル</t>
+          <t>【飛田新地】思い出を形に残す写真旅！カメラや旅行趣味を楽しむ現役キャストのライフスタイル</t>
         </is>
       </c>
       <c r="C87" s="9" t="inlineStr">
@@ -5150,7 +5150,7 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】アロマで心身リラックス！お仕事終わりのお部屋を満たす香りのリフレッシュ習慣</t>
+          <t>【飛田新地】アロマで心身リラックス！お仕事終わりのお部屋を満たす香りのリフレッシュ習慣</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -5203,7 +5203,7 @@
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】ふわふわパンケーキで極上カフェタイム！休日に味わう自分への甘いご褒美</t>
+          <t>【飛田新地】ふわふわパンケーキで極上カフェタイム！休日に味わう自分への甘いご褒美</t>
         </is>
       </c>
       <c r="C89" s="9" t="inlineStr">
@@ -5256,7 +5256,7 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】和装の帯結び・リボンアレンジ！料亭で一目置かれる上品な和装コーディネート</t>
+          <t>【飛田新地】和装の帯結び・リボンアレンジ！料亭で一目置かれる上品な和装コーディネート</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -5309,7 +5309,7 @@
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】貯金箱がどんどん溜まる！半年で100万円貯めるための現実的なステップ</t>
+          <t>【飛田新地】貯金箱がどんどん溜まる！半年で100万円貯めるための現実的なステップ</t>
         </is>
       </c>
       <c r="C91" s="9" t="inlineStr">
@@ -5362,7 +5362,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】ハーブティーでほっと一息！お仕事終わりに試したいオーガニック温活習慣</t>
+          <t>【飛田新地】ハーブティーでほっと一息！お仕事終わりに試したいオーガニック温活習慣</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】スキンケア見直し術！毎日のメイク映えを叶える透明感美肌のつくり方</t>
+          <t>【飛田新地】スキンケア見直し術！毎日のメイク映えを叶える透明感美肌のつくり方</t>
         </is>
       </c>
       <c r="C93" s="9" t="inlineStr">
@@ -5468,7 +5468,7 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】ぬくもり溢れるお部屋づくり！ふんわり毛布と間接照明で最高の癒やし空間</t>
+          <t>【飛田新地】ぬくもり溢れるお部屋づくり！ふんわり毛布と間接照明で最高の癒やし空間</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -5521,7 +5521,7 @@
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】夢を叶える手帳術！目標額・欲しいものリストを書いてモチベーションUP</t>
+          <t>【飛田新地】夢を叶える手帳術！目標額・欲しいものリストを書いてモチベーションUP</t>
         </is>
       </c>
       <c r="C95" s="9" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】お酒不要！ノンアルドリンク！乾杯シーンでも可愛くスマートに魅せるコツ</t>
+          <t>【飛田新地】お酒不要！ノンアルドリンク！乾杯シーンでも可愛くスマートに魅せるコツ</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】足湯＆フットケア！一日頑張った足を労わる自宅でできるリフレッシュ</t>
+          <t>【飛田新地】足湯＆フットケア！一日頑張った足を労わる自宅でできるリフレッシュ</t>
         </is>
       </c>
       <c r="C97" s="9" t="inlineStr">
@@ -5680,7 +5680,7 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】星モチーフアクセサリー！首元でキラリと光るシンプルジュエリーの魅力</t>
+          <t>【飛田新地】星モチーフアクセサリー！首元でキラリと光るシンプルジュエリーの魅力</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -5733,7 +5733,7 @@
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】悪質スカウト・反社排除！SNS求人の罠とヤクザ店舗の危険性！直営グループ応募が安全な理由</t>
+          <t>【飛田新地】悪質スカウト・反社排除！SNS求人の罠とヤクザ店舗の危険性！直営グループ応募が安全な理由</t>
         </is>
       </c>
       <c r="C99" s="9" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】悪質店舗の見極め方！日給保証の嘘・雑費天引き・罰金ペナルティを課す要注意店舗の3大特徴</t>
+          <t>【飛田新地】悪質店舗の見極め方！日給保証の嘘・雑費天引き・罰金ペナルティを課す要注意店舗の3大特徴</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -5839,7 +5839,7 @@
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>【飛田新地 求人】シンママ・子育て支援！提携託児所完備＆短時間シフト！ママさんが安心して高収入を得る方法</t>
+          <t>【飛田新地】シンママ・子育て支援！提携託児所完備＆短時間シフト！ママさんが安心して高収入を得る方法</t>
         </is>
       </c>
       <c r="C101" s="9" t="inlineStr">

</xml_diff>